<commit_message>
WIP: data update test
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Downloads\90in90\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gyzl-my.sharepoint.com/personal/sikudova_gymzl_cz/Documents/90mistza90dni/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE0868CA-6A3A-41E9-A94B-ED9D2B1014B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{AE0868CA-6A3A-41E9-A94B-ED9D2B1014B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F390EFA2-650B-4725-86A7-29B9C69907C4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="71">
   <si>
     <t>Navštívené místo</t>
   </si>
@@ -251,6 +251,12 @@
   </si>
   <si>
     <t>(prázdné)</t>
+  </si>
+  <si>
+    <t>19: nedostavěná Baťova dálnice (mostek)</t>
+  </si>
+  <si>
+    <t>84: Brdo</t>
   </si>
 </sst>
 </file>
@@ -608,7 +614,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90B89549-8DEE-4BD2-A477-2CC98B007387}">
-  <dimension ref="A1:M58"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="58.33203125" bestFit="1" customWidth="1"/>
@@ -736,8 +742,11 @@
       <c r="H5">
         <v>1</v>
       </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
       <c r="M5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
@@ -834,11 +843,14 @@
       <c r="A12" t="s">
         <v>21</v>
       </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
       <c r="F12">
         <v>1</v>
       </c>
       <c r="M12">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -885,24 +897,18 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="K16">
-        <v>1</v>
-      </c>
       <c r="M16">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -910,10 +916,10 @@
       <c r="D17">
         <v>1</v>
       </c>
-      <c r="H17">
-        <v>1</v>
-      </c>
-      <c r="J17">
+      <c r="K17">
+        <v>1</v>
+      </c>
+      <c r="L17">
         <v>1</v>
       </c>
       <c r="M17">
@@ -922,7 +928,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -930,41 +936,47 @@
       <c r="D18">
         <v>1</v>
       </c>
-      <c r="F18">
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="J18">
         <v>1</v>
       </c>
       <c r="M18">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
       </c>
       <c r="D19">
         <v>1</v>
       </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
       <c r="M19">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="D20">
         <v>1</v>
       </c>
       <c r="M20">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -972,16 +984,13 @@
       <c r="D21">
         <v>1</v>
       </c>
-      <c r="F21">
-        <v>1</v>
-      </c>
       <c r="M21">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B22">
         <v>1</v>
@@ -989,7 +998,7 @@
       <c r="D22">
         <v>1</v>
       </c>
-      <c r="H22">
+      <c r="F22">
         <v>1</v>
       </c>
       <c r="M22">
@@ -998,18 +1007,24 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
       <c r="M23">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B24">
         <v>1</v>
@@ -1020,7 +1035,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25">
         <v>1</v>
@@ -1031,24 +1046,18 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
-      <c r="D26">
-        <v>1</v>
-      </c>
-      <c r="L26">
-        <v>1</v>
-      </c>
       <c r="M26">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B27">
         <v>1</v>
@@ -1065,18 +1074,24 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
       </c>
       <c r="D28">
         <v>1</v>
       </c>
+      <c r="L28">
+        <v>1</v>
+      </c>
       <c r="M28">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -1087,7 +1102,7 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -1098,7 +1113,7 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D31">
         <v>1</v>
@@ -1109,53 +1124,56 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B32">
         <v>1</v>
       </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
       <c r="M32">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B33">
         <v>1</v>
       </c>
-      <c r="D33">
-        <v>1</v>
-      </c>
-      <c r="F33">
-        <v>1</v>
-      </c>
       <c r="M33">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>62</v>
+        <v>42</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+      <c r="M34">
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>43</v>
-      </c>
-      <c r="B35">
-        <v>1</v>
-      </c>
-      <c r="M35">
-        <v>1</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>44</v>
-      </c>
-      <c r="D36">
+        <v>43</v>
+      </c>
+      <c r="B36">
         <v>1</v>
       </c>
       <c r="M36">
@@ -1164,9 +1182,9 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>45</v>
-      </c>
-      <c r="B37">
+        <v>44</v>
+      </c>
+      <c r="D37">
         <v>1</v>
       </c>
       <c r="M37">
@@ -1175,30 +1193,18 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B38">
         <v>1</v>
       </c>
-      <c r="D38">
-        <v>1</v>
-      </c>
-      <c r="F38">
-        <v>1</v>
-      </c>
-      <c r="I38">
-        <v>1</v>
-      </c>
-      <c r="J38">
-        <v>1</v>
-      </c>
       <c r="M38">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B39">
         <v>1</v>
@@ -1206,13 +1212,22 @@
       <c r="D39">
         <v>1</v>
       </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="I39">
+        <v>1</v>
+      </c>
+      <c r="J39">
+        <v>1</v>
+      </c>
       <c r="M39">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B40">
         <v>1</v>
@@ -1220,16 +1235,13 @@
       <c r="D40">
         <v>1</v>
       </c>
-      <c r="K40">
-        <v>1</v>
-      </c>
       <c r="M40">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B41">
         <v>1</v>
@@ -1237,7 +1249,7 @@
       <c r="D41">
         <v>1</v>
       </c>
-      <c r="J41">
+      <c r="K41">
         <v>1</v>
       </c>
       <c r="M41">
@@ -1246,20 +1258,26 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
       </c>
       <c r="D42">
         <v>1</v>
       </c>
+      <c r="J42">
+        <v>1</v>
+      </c>
       <c r="M42">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>51</v>
-      </c>
-      <c r="F43">
+        <v>50</v>
+      </c>
+      <c r="D43">
         <v>1</v>
       </c>
       <c r="M43">
@@ -1268,9 +1286,9 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>52</v>
-      </c>
-      <c r="E44">
+        <v>51</v>
+      </c>
+      <c r="F44">
         <v>1</v>
       </c>
       <c r="M44">
@@ -1279,32 +1297,32 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>53</v>
-      </c>
-      <c r="B45">
-        <v>1</v>
-      </c>
-      <c r="L45">
+        <v>52</v>
+      </c>
+      <c r="E45">
         <v>1</v>
       </c>
       <c r="M45">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>54</v>
-      </c>
-      <c r="D46">
+        <v>53</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="L46">
         <v>1</v>
       </c>
       <c r="M46">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="D47">
         <v>1</v>
@@ -1315,35 +1333,35 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>55</v>
-      </c>
-      <c r="C48">
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="D48">
         <v>1</v>
       </c>
-      <c r="J48">
-        <v>1</v>
-      </c>
       <c r="M48">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>65</v>
+        <v>55</v>
+      </c>
+      <c r="C49">
+        <v>1</v>
       </c>
       <c r="D49">
         <v>1</v>
       </c>
+      <c r="J49">
+        <v>1</v>
+      </c>
       <c r="M49">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D50">
         <v>1</v>
@@ -1354,7 +1372,7 @@
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D51">
         <v>1</v>
@@ -1365,35 +1383,29 @@
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>56</v>
-      </c>
-      <c r="D52">
-        <v>1</v>
-      </c>
-      <c r="H52">
+        <v>70</v>
+      </c>
+      <c r="B52">
         <v>1</v>
       </c>
       <c r="M52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>57</v>
-      </c>
-      <c r="B53">
-        <v>1</v>
-      </c>
-      <c r="F53">
+        <v>67</v>
+      </c>
+      <c r="D53">
         <v>1</v>
       </c>
       <c r="M53">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D54">
         <v>1</v>
@@ -1407,70 +1419,98 @@
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B55">
         <v>1</v>
       </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
       <c r="M55">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>60</v>
-      </c>
-      <c r="B56">
+        <v>58</v>
+      </c>
+      <c r="D56">
+        <v>1</v>
+      </c>
+      <c r="H56">
         <v>1</v>
       </c>
       <c r="M56">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>68</v>
+        <v>59</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+      <c r="M57">
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+      <c r="M58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
         <v>11</v>
       </c>
-      <c r="B58">
-        <v>34</v>
-      </c>
-      <c r="C58">
-        <v>1</v>
-      </c>
-      <c r="D58">
-        <v>36</v>
-      </c>
-      <c r="E58">
+      <c r="B60">
+        <v>37</v>
+      </c>
+      <c r="C60">
+        <v>1</v>
+      </c>
+      <c r="D60">
+        <v>37</v>
+      </c>
+      <c r="E60">
         <v>2</v>
       </c>
-      <c r="F58">
+      <c r="F60">
         <v>14</v>
       </c>
-      <c r="G58">
-        <v>1</v>
-      </c>
-      <c r="H58">
+      <c r="G60">
+        <v>1</v>
+      </c>
+      <c r="H60">
         <v>10</v>
       </c>
-      <c r="I58">
-        <v>1</v>
-      </c>
-      <c r="J58">
+      <c r="I60">
+        <v>1</v>
+      </c>
+      <c r="J60">
         <v>4</v>
       </c>
-      <c r="K58">
+      <c r="K60">
         <v>2</v>
       </c>
-      <c r="L58">
-        <v>3</v>
-      </c>
-      <c r="M58">
-        <v>108</v>
+      <c r="L60">
+        <v>5</v>
+      </c>
+      <c r="M60">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>